<commit_message>
feat: add launch configuration and project documentation resources
</commit_message>
<xml_diff>
--- a/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
+++ b/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_20E8D5C66FBEC0ADF70C915E712B6542735C97F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F11B3316-C315-4814-8220-F103964EB436}"/>
   <bookViews>
-    <workbookView xWindow="-12" yWindow="-12" windowWidth="6036" windowHeight="4560"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -68,7 +74,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="5" formatCode="#,##0\ &quot;€&quot;;\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
@@ -279,7 +285,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -288,9 +294,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -376,7 +379,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Euro" xfId="1"/>
+    <cellStyle name="Euro" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
   </cellStyles>
@@ -386,12 +389,15 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -473,9 +479,20 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1270</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1126</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2F8A-4B88-8C56-501CB47914E0}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -529,9 +546,20 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1374</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>786</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2F8A-4B88-8C56-501CB47914E0}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -588,6 +616,11 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-2F8A-4B88-8C56-501CB47914E0}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -761,7 +794,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -843,9 +876,20 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.41499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7F29-406F-AB04-1BEDB655BA0B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -899,9 +943,20 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.80900000000000005</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-7F29-406F-AB04-1BEDB655BA0B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -958,6 +1013,11 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-7F29-406F-AB04-1BEDB655BA0B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -1031,7 +1091,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
-          <c:min val="0.7"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1131,7 +1191,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -1213,9 +1273,20 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.61799999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.75</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-ABE0-4A44-B531-C1467FCE67D1}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1269,9 +1340,20 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.53600000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.67</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-ABE0-4A44-B531-C1467FCE67D1}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -1328,6 +1410,11 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-ABE0-4A44-B531-C1467FCE67D1}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -1400,8 +1487,8 @@
         <c:axId val="114876800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="1"/>
-          <c:min val="0.6"/>
+          <c:max val="0.70000000000000007"/>
+          <c:min val="0.2"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1517,7 +1604,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="16385" name="Graphique 1"/>
+        <xdr:cNvPr id="16385" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001400000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -1549,7 +1642,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="16386" name="Graphique 2"/>
+        <xdr:cNvPr id="16386" name="Graphique 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002400000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -1581,7 +1680,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="16387" name="Graphique 3"/>
+        <xdr:cNvPr id="16387" name="Graphique 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003400000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -1618,7 +1723,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7171" name="Rectangle 3"/>
+        <xdr:cNvPr id="7171" name="Rectangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000031C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeArrowheads="1"/>
         </xdr:cNvSpPr>
@@ -1680,7 +1791,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7172" name="Rectangle 4"/>
+        <xdr:cNvPr id="7172" name="Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000041C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeArrowheads="1"/>
         </xdr:cNvSpPr>
@@ -1742,7 +1859,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7173" name="Rectangle 5"/>
+        <xdr:cNvPr id="7173" name="Rectangle 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000051C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeArrowheads="1"/>
         </xdr:cNvSpPr>
@@ -1807,7 +1930,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7175" name="AutoShape 7"/>
+        <xdr:cNvPr id="7175" name="AutoShape 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000071C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks/>
         </xdr:cNvSpPr>
@@ -1860,7 +1989,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7176" name="AutoShape 8"/>
+        <xdr:cNvPr id="7176" name="AutoShape 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000081C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks/>
         </xdr:cNvSpPr>
@@ -1913,7 +2048,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7177" name="AutoShape 9"/>
+        <xdr:cNvPr id="7177" name="AutoShape 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-0000091C0000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks/>
         </xdr:cNvSpPr>
@@ -1952,6 +2093,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2325,220 +2470,220 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46875" defaultRowHeight="12.7" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="9" width="14.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="9" width="14.3515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.64453125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.46875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="27" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="28"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="24" t="s">
+      <c r="E1" s="27"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="25"/>
-      <c r="I1" s="26"/>
-    </row>
-    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="24"/>
+      <c r="I1" s="25"/>
+    </row>
+    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="4"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="4"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H2" s="2"/>
+      <c r="I2" s="4"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="4"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="5"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="4"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H3" s="2"/>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="5"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="5"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="4"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="5"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="2"/>
+      <c r="I4" s="4"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="4"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="5"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="4"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="5"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H5" s="2"/>
+      <c r="I5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="5"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="4"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="5"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="4"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="5"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H6" s="2"/>
+      <c r="I6" s="4"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="5"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="4"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="5"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="4"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="2"/>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="5"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="4"/>
       <c r="D8" s="3"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="5"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="4"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="5"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H8" s="2"/>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="5"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="4"/>
       <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="5"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="4"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="5"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="2"/>
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="5"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="3"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="5"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="4"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="5"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H10" s="2"/>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="5"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="4"/>
       <c r="D11" s="3"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="5"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="4"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="5"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="2"/>
+      <c r="I11" s="4"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="5"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="4"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="4"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="5"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H12" s="2"/>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="5"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="4"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="5"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="4"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="5"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H13" s="2"/>
+      <c r="I13" s="4"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="5"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="4"/>
       <c r="D14" s="3"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="5"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="4"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="5"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H14" s="2"/>
+      <c r="I14" s="4"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="5"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="4"/>
       <c r="D15" s="3"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="5"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="4"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="5"/>
-    </row>
-    <row r="16" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H15" s="2"/>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="5"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="4"/>
       <c r="D16" s="3"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="5"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="4"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="5"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H16" s="2"/>
+      <c r="I16" s="4"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="5"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="4"/>
       <c r="D17" s="3"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="4"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="5"/>
-    </row>
-    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="8"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H17" s="2"/>
+      <c r="I17" s="4"/>
+    </row>
+    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2549,8 +2694,8 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="23" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A23" s="22" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2569,162 +2714,186 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46875" defaultRowHeight="12.7" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="27.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="1" width="27.52734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.87890625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.46875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="B3" s="10">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0</v>
+      </c>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="B4" s="12">
+        <v>0.80900000000000005</v>
+      </c>
+      <c r="C4" s="12">
+        <v>0</v>
+      </c>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+    </row>
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-    </row>
-    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="B8" s="10">
+        <v>0.61799999999999999</v>
+      </c>
+      <c r="C8" s="10">
+        <v>0.75</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+    </row>
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B9" s="12">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="C9" s="12">
+        <v>0.67</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+    </row>
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="16" t="s">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+    </row>
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-    </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="B14" s="16">
+        <v>1270</v>
+      </c>
+      <c r="C14" s="17">
+        <v>1126</v>
+      </c>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+    </row>
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-    </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="B15" s="18">
+        <v>1374</v>
+      </c>
+      <c r="C15" s="19">
+        <v>786</v>
+      </c>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+    </row>
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
     </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>

</xml_diff>

<commit_message>
Please provide the diff or the list of changes you would like summarized.
</commit_message>
<xml_diff>
--- a/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
+++ b/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_20E8D5C66FBEC0ADF70C915E712B6542735C97F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F11B3316-C315-4814-8220-F103964EB436}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_20E8D5C66FBEC0ADF70C915E712B6542735C97F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E58CF7A-FE8C-4C92-A897-7CF28004A422}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -480,10 +480,10 @@
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1270</c:v>
+                  <c:v>1123</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1126</c:v>
+                  <c:v>965</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -547,10 +547,10 @@
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1374</c:v>
+                  <c:v>2013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>786</c:v>
+                  <c:v>1665</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -877,7 +877,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.41499999999999998</c:v>
+                  <c:v>0.56000000000000005</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -944,10 +944,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.80900000000000005</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.76300000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1274,10 +1274,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.61799999999999999</c:v>
+                  <c:v>0.57509999999999994</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.75</c:v>
+                  <c:v>0.76729999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1341,10 +1341,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.53600000000000003</c:v>
+                  <c:v>0.73719999999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.67</c:v>
+                  <c:v>0.71</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1487,7 +1487,7 @@
         <c:axId val="114876800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="0.70000000000000007"/>
+          <c:max val="0.9"/>
           <c:min val="0.2"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -2472,14 +2472,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46875" defaultRowHeight="12.7" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46484375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="9" width="14.3515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.64453125" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.46875" style="1"/>
+    <col min="1" max="9" width="14.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.46484375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
         <v>10</v>
       </c>
@@ -2496,7 +2496,7 @@
       <c r="H1" s="24"/>
       <c r="I1" s="25"/>
     </row>
-    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="2"/>
       <c r="C2" s="4"/>
@@ -2507,7 +2507,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="2"/>
       <c r="C3" s="4"/>
@@ -2518,7 +2518,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
       <c r="B4" s="2"/>
       <c r="C4" s="4"/>
@@ -2529,7 +2529,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="2"/>
       <c r="C5" s="4"/>
@@ -2540,7 +2540,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="2"/>
       <c r="C6" s="4"/>
@@ -2551,7 +2551,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="2"/>
       <c r="C7" s="4"/>
@@ -2562,7 +2562,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="2"/>
       <c r="C8" s="4"/>
@@ -2573,7 +2573,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
       <c r="B9" s="2"/>
       <c r="C9" s="4"/>
@@ -2584,7 +2584,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="2"/>
       <c r="C10" s="4"/>
@@ -2595,7 +2595,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="2"/>
       <c r="C11" s="4"/>
@@ -2606,7 +2606,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="2"/>
       <c r="C12" s="4"/>
@@ -2617,7 +2617,7 @@
       <c r="H12" s="2"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="2"/>
       <c r="C13" s="4"/>
@@ -2628,7 +2628,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="2"/>
       <c r="C14" s="4"/>
@@ -2639,7 +2639,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="2"/>
       <c r="C15" s="4"/>
@@ -2650,7 +2650,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="2"/>
       <c r="C16" s="4"/>
@@ -2661,7 +2661,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="4"/>
@@ -2672,7 +2672,7 @@
       <c r="H17" s="2"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
@@ -2683,7 +2683,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="7"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2694,7 +2694,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="22" t="s">
         <v>15</v>
       </c>
@@ -2716,14 +2716,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46875" defaultRowHeight="12.7" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46484375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.52734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.87890625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.46875" style="1"/>
+    <col min="1" max="1" width="27.53125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.46484375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -2740,12 +2740,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="10">
-        <v>0.41499999999999998</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="C3" s="10">
         <v>0</v>
@@ -2753,20 +2753,20 @@
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="12">
-        <v>0.80900000000000005</v>
+        <v>1</v>
       </c>
       <c r="C4" s="12">
-        <v>0</v>
+        <v>0.76300000000000001</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
     </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
@@ -2775,8 +2775,8 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
     </row>
-    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
@@ -2793,33 +2793,33 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="10">
-        <v>0.61799999999999999</v>
+        <v>0.57509999999999994</v>
       </c>
       <c r="C8" s="10">
-        <v>0.75</v>
+        <v>0.76729999999999998</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
     </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="12">
-        <v>0.53600000000000003</v>
+        <v>0.73719999999999997</v>
       </c>
       <c r="C9" s="12">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
     </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>5</v>
       </c>
@@ -2828,8 +2828,8 @@
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
     </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="15" t="s">
         <v>2</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>1</v>
       </c>
@@ -2860,33 +2860,33 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B14" s="16">
-        <v>1270</v>
+        <v>1123</v>
       </c>
       <c r="C14" s="17">
-        <v>1126</v>
+        <v>965</v>
       </c>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
     </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B15" s="18">
-        <v>1374</v>
+        <v>2013</v>
       </c>
       <c r="C15" s="19">
-        <v>786</v>
+        <v>1665</v>
       </c>
       <c r="D15" s="19"/>
       <c r="E15" s="19"/>
     </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
feat: add training materials and industrial organization documentation for TI18 session
</commit_message>
<xml_diff>
--- a/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
+++ b/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/Tableau de bord.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/jeu_du_kanban/clé USB Jeu du Kanban/Animation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_20E8D5C66FBEC0ADF70C915E712B6542735C97F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E58CF7A-FE8C-4C92-A897-7CF28004A422}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_20E8D5C66FBEC0ADF70C915E712B6542735C97F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F5C3430-1326-4388-AC97-9E78D0D73092}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="19440" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -480,10 +480,7 @@
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1123</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>965</c:v>
+                  <c:v>720</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -547,10 +544,7 @@
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2013</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1665</c:v>
+                  <c:v>1166</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -613,6 +607,9 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1238</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -877,10 +874,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.56000000000000005</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.62</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -944,10 +938,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.76300000000000001</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1010,6 +1001,9 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.4</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1274,10 +1268,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.57509999999999994</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.76729999999999998</c:v>
+                  <c:v>0.60699999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1341,10 +1332,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.73719999999999997</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.71</c:v>
+                  <c:v>0.624</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1407,6 +1395,9 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.68799999999999994</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2095,10 +2086,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -2745,11 +2732,9 @@
         <v>3</v>
       </c>
       <c r="B3" s="10">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="C3" s="10">
-        <v>0</v>
-      </c>
+        <v>0.62</v>
+      </c>
+      <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
     </row>
@@ -2758,11 +2743,9 @@
         <v>4</v>
       </c>
       <c r="B4" s="12">
-        <v>1</v>
-      </c>
-      <c r="C4" s="12">
-        <v>0.76300000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C4" s="12"/>
       <c r="D4" s="12"/>
       <c r="E4" s="12"/>
     </row>
@@ -2770,7 +2753,9 @@
       <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="14">
+        <v>0.4</v>
+      </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
@@ -2798,11 +2783,9 @@
         <v>3</v>
       </c>
       <c r="B8" s="10">
-        <v>0.57509999999999994</v>
-      </c>
-      <c r="C8" s="10">
-        <v>0.76729999999999998</v>
-      </c>
+        <v>0.60699999999999998</v>
+      </c>
+      <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
     </row>
@@ -2811,11 +2794,9 @@
         <v>4</v>
       </c>
       <c r="B9" s="12">
-        <v>0.73719999999999997</v>
-      </c>
-      <c r="C9" s="12">
-        <v>0.71</v>
-      </c>
+        <v>0.624</v>
+      </c>
+      <c r="C9" s="12"/>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
     </row>
@@ -2823,7 +2804,9 @@
       <c r="A10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="14">
+        <v>0.68799999999999994</v>
+      </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
@@ -2865,11 +2848,9 @@
         <v>3</v>
       </c>
       <c r="B14" s="16">
-        <v>1123</v>
-      </c>
-      <c r="C14" s="17">
-        <v>965</v>
-      </c>
+        <v>720</v>
+      </c>
+      <c r="C14" s="17"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
     </row>
@@ -2878,11 +2859,9 @@
         <v>4</v>
       </c>
       <c r="B15" s="18">
-        <v>2013</v>
-      </c>
-      <c r="C15" s="19">
-        <v>1665</v>
-      </c>
+        <v>1166</v>
+      </c>
+      <c r="C15" s="19"/>
       <c r="D15" s="19"/>
       <c r="E15" s="19"/>
     </row>
@@ -2890,7 +2869,9 @@
       <c r="A16" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="20"/>
+      <c r="B16" s="20">
+        <v>1238</v>
+      </c>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>

</xml_diff>